<commit_message>
change in the file manager
</commit_message>
<xml_diff>
--- a/uploads/blockade-quiz-questions.xlsx
+++ b/uploads/blockade-quiz-questions.xlsx
@@ -421,39 +421,39 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>বঙ্গবন্ধু শেখ মুজিবুর রহমান কৃষি বিশ্ববিদ্যালয়টি কোথায় অবস্থিত?</v>
+        <v>কৃষি তথ্য সংস্থা আত্মপ্রকাশ করে কত সালে?</v>
       </c>
       <c r="B2" t="str">
-        <v>ঢাকা</v>
+        <v>১৯৫০</v>
       </c>
       <c r="C2" t="str">
-        <v>গাজীপুর</v>
+        <v>১৯৫৬</v>
       </c>
       <c r="D2" t="str">
-        <v>ময়মনসিংহ</v>
+        <v>১৯৬১</v>
       </c>
       <c r="E2" t="str">
-        <v>সিলেট</v>
+        <v>১৯৬৫</v>
       </c>
       <c r="F2" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>নিচের কোনটি উদ্যান ফসল?</v>
+        <v>BRRI এর প্রধান কার্যালয় কোথায়?</v>
       </c>
       <c r="B3" t="str">
-        <v>তুলা</v>
+        <v>রাজশাহী</v>
       </c>
       <c r="C3" t="str">
-        <v>ধান</v>
+        <v>দিনাজপুর</v>
       </c>
       <c r="D3" t="str">
-        <v>পাট</v>
+        <v>ময়মনসিংহ</v>
       </c>
       <c r="E3" t="str">
-        <v>গোল আলু</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="F3" t="str">
         <v>D</v>
@@ -461,19 +461,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>অভ্যন্তরীণ জলাশয়ের মধ্যে নিচের কোনটির আয়তন সবচেয়ে কম ?</v>
+        <v>হাজী মোহাম্মদ দানেশ বিজ্ঞান ও প্রযুক্তি বিশ্ববিদ্যালয় কোন জেলায় অবস্থিত?</v>
       </c>
       <c r="B4" t="str">
-        <v>পুকুর ডোবা</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="C4" t="str">
-        <v>বাঁওড়</v>
+        <v>দিনাজপুর</v>
       </c>
       <c r="D4" t="str">
-        <v>বিল</v>
+        <v>ময়মনসিংহ</v>
       </c>
       <c r="E4" t="str">
-        <v>চিংড়ি খামার</v>
+        <v>রাজশাহী</v>
       </c>
       <c r="F4" t="str">
         <v>B</v>
@@ -481,19 +481,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>বাংলাদেশে সর্বাধিক সংখ্যক উন্নত জাতের ধান উদ্ভাবক প্রতিষ্ঠান</v>
+        <v>নিচের কোনটি দানাজাতীয় ফসল?</v>
       </c>
       <c r="B5" t="str">
-        <v>BAU</v>
+        <v>সূর্যমুখী</v>
       </c>
       <c r="C5" t="str">
-        <v>BRRI</v>
+        <v>কাউন</v>
       </c>
       <c r="D5" t="str">
-        <v>BINA</v>
+        <v>শনপাট</v>
       </c>
       <c r="E5" t="str">
-        <v>BARI</v>
+        <v>মেস্তা</v>
       </c>
       <c r="F5" t="str">
         <v>B</v>
@@ -501,19 +501,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>বাংলাদেশ পরমাণু কৃষি গবেষণা কোথায় অবস্থিত?</v>
+        <v>কৃষির ইংরেজিতে Agriculture শব্দটি এসেছে-</v>
       </c>
       <c r="B6" t="str">
-        <v>ময়মনসিংহ</v>
+        <v>ল্যাটিন শব্দ হতে</v>
       </c>
       <c r="C6" t="str">
-        <v>জামালপুর</v>
+        <v>ব্রিটিশ শব্দ হতে</v>
       </c>
       <c r="D6" t="str">
-        <v>জয়দেবপুর</v>
+        <v>ফারসি শব্দ হতে</v>
       </c>
       <c r="E6" t="str">
-        <v>হবিগঞ্জ</v>
+        <v>চৈনিক শব্দ হতে</v>
       </c>
       <c r="F6" t="str">
         <v>A</v>
@@ -521,39 +521,39 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>কৃষি উপকরণ সরবরাহকারী সরকারি প্রতিষ্ঠান কোনটি?</v>
+        <v>নিচের কোন ফসলটি বেশি যত্নে চাষ করা হয়?</v>
       </c>
       <c r="B7" t="str">
-        <v>বিএডিসি</v>
+        <v>গম</v>
       </c>
       <c r="C7" t="str">
-        <v>কৃষি তথ্য সার্ভিস</v>
+        <v>পাট</v>
       </c>
       <c r="D7" t="str">
-        <v>ডি এই</v>
+        <v>টমেটো</v>
       </c>
       <c r="E7" t="str">
-        <v>বি আর আই</v>
+        <v>ইক্ষু</v>
       </c>
       <c r="F7" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>বাংলাদেশ ধান গবেষণা ইনস্টিটিউট কোথায় অবস্থিত?</v>
+        <v>নিচের কোনটি পানীয় ফসল?</v>
       </c>
       <c r="B8" t="str">
-        <v>ঢাকা</v>
+        <v>তামাক</v>
       </c>
       <c r="C8" t="str">
-        <v>গাজীপুর</v>
+        <v>চা</v>
       </c>
       <c r="D8" t="str">
-        <v>দিনাজপুর</v>
+        <v>সরগম</v>
       </c>
       <c r="E8" t="str">
-        <v>পঞ্চগড়</v>
+        <v>চিনা</v>
       </c>
       <c r="F8" t="str">
         <v>B</v>
@@ -561,79 +561,79 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BRAC কত সালে প্রতিষ্ঠিত হয়?</v>
+        <v>নিচের কোনটি বদ্ধ জলাশয়ের উদাহরণ?</v>
       </c>
       <c r="B9" t="str">
-        <v>১৯৭০</v>
+        <v>নদী</v>
       </c>
       <c r="C9" t="str">
-        <v>১৯৭১</v>
+        <v>খাল</v>
       </c>
       <c r="D9" t="str">
-        <v>১৯৭২</v>
+        <v>হাওর</v>
       </c>
       <c r="E9" t="str">
-        <v>১৯৭৩</v>
+        <v>বাঁওর</v>
       </c>
       <c r="F9" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>কৃষি শিক্ষক দুটি বিষয় নিয়ে বেশি আলোচনার কারণ কোনটি?</v>
+        <v>মানুষের মৌলিক চাহিদার দ্বিতীয় উপকরণটি কী?</v>
       </c>
       <c r="B10" t="str">
-        <v>প্রধান খাদ্য</v>
+        <v>খাদ্য</v>
       </c>
       <c r="C10" t="str">
-        <v>অর্থনৈতিক গুরুত্ব</v>
+        <v>চিকিৎসা</v>
       </c>
       <c r="D10" t="str">
-        <v>পুষ্টির চাহিদা পূরণ</v>
+        <v>বস্তু</v>
       </c>
       <c r="E10" t="str">
-        <v>উৎপাদন ঝুঁকি</v>
+        <v>শিক্ষা</v>
       </c>
       <c r="F10" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>নিচের কোন প্রতিষ্ঠান কৃষক সভার আয়োজন করে?</v>
+        <v>কৃষির প্রধান ক্ষেত্র-</v>
       </c>
       <c r="B11" t="str">
-        <v>কৃষি সম্প্রসারণ অধিদপ্তর</v>
+        <v>২ টি</v>
       </c>
       <c r="C11" t="str">
-        <v>বাংলাদেশ কৃষি উন্নয়ন কর্পোরেশন</v>
+        <v>৪ টি</v>
       </c>
       <c r="D11" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা কাউন্সিল</v>
+        <v>৬ টি</v>
       </c>
       <c r="E11" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট</v>
+        <v>৮ টি</v>
       </c>
       <c r="F11" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>নিচের কোনটি দানা জাতীয় ফসল?</v>
+        <v>নিচের কোনটি উদ্যান ফসল ?</v>
       </c>
       <c r="B12" t="str">
-        <v>ছোলা</v>
+        <v>তুলা</v>
       </c>
       <c r="C12" t="str">
-        <v>সরিষা</v>
+        <v>&lt;p&gt;ধান&lt;/p&gt;</v>
       </c>
       <c r="D12" t="str">
-        <v>চীনাবাদাম</v>
+        <v>&lt;p&gt;পাট&lt;/p&gt;</v>
       </c>
       <c r="E12" t="str">
-        <v>ধান</v>
+        <v>&lt;p&gt;গোল আলু&lt;/p&gt;</v>
       </c>
       <c r="F12" t="str">
         <v>D</v>
@@ -641,179 +641,179 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>পাটকে মাঠ ফসল বলা কারণ-</v>
+        <v>নিচের কোনটি মাঠ ফসল।</v>
       </c>
       <c r="B13" t="str">
-        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
+        <v>পিঁয়াজ</v>
       </c>
       <c r="C13" t="str">
-        <v>ফসলের লাভ ও ব্যয়ের অনুপাত বেশি হয়</v>
+        <v>ভুট্টা</v>
       </c>
       <c r="D13" t="str">
-        <v>সমস্ত ফসল একত্রে পরিপক্ক ও সংগ্রহ করা হয়</v>
+        <v>টমেটো</v>
       </c>
       <c r="E13" t="str">
-        <v>ফসলের মূল্য মৌসুমের শুরুতে বেশি হয়</v>
+        <v>আম</v>
       </c>
       <c r="F13" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>BARI কোথায় অবস্থিত?</v>
+        <v>কতভাগ জমিতে উদ্যান ফসলের চাষ হয়?</v>
       </c>
       <c r="B14" t="str">
-        <v>ময়মনসিংহ</v>
+        <v>৭০ ভাগ</v>
       </c>
       <c r="C14" t="str">
-        <v>গাজীপুর</v>
+        <v>৫০ ভাগ</v>
       </c>
       <c r="D14" t="str">
-        <v>সাভার</v>
+        <v>৩০ ভাগ</v>
       </c>
       <c r="E14" t="str">
-        <v>সিলেট</v>
+        <v>১৪ ভাগ</v>
       </c>
       <c r="F14" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>স্থানীয় 'কৃষি তথ্য ভাণ্ডার' বলা হয় কাকে?</v>
+        <v>নিচের কোনটি সবুজ সার জাতীয় ফসল?</v>
       </c>
       <c r="B15" t="str">
-        <v>সাধারণ কৃষক</v>
+        <v>চীনা</v>
       </c>
       <c r="C15" t="str">
-        <v>অভিজ্ঞ কৃষক</v>
+        <v>কফি</v>
       </c>
       <c r="D15" t="str">
-        <v>বয়স্ক কৃষক</v>
+        <v>শণপাট</v>
       </c>
       <c r="E15" t="str">
-        <v>কৃষক সভা</v>
+        <v>তিল</v>
       </c>
       <c r="F15" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ফসলের নতুন নতুন জাত উদ্ভাবন ও উন্নয়ন সাধনের কাজ করে নিচের কোন প্রতিষ্ঠানটি?</v>
+        <v>একটি কৃষক সভায় অংশগ্রহণকারী সদস্যের সংখ্যা সাধারণত কত?</v>
       </c>
       <c r="B16" t="str">
-        <v>BARI</v>
+        <v>২০-৩০ জন</v>
       </c>
       <c r="C16" t="str">
-        <v>BINA</v>
+        <v>২৫-৩০ জন</v>
       </c>
       <c r="D16" t="str">
-        <v>BARC</v>
+        <v>৩০-৪০ জন</v>
       </c>
       <c r="E16" t="str">
-        <v>BRRI</v>
+        <v>৫০-৬০ জন</v>
       </c>
       <c r="F16" t="str">
-        <v>A</v>
+        <v>D</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>মানুষের মৌলিক চাহিদার দ্বিতীয় উপকরণটি কী?</v>
+        <v>নিচের কোনটি উদ্যান ফসল?</v>
       </c>
       <c r="B17" t="str">
-        <v>খাদ্য</v>
+        <v>তুলা</v>
       </c>
       <c r="C17" t="str">
-        <v>চিকিৎসা</v>
+        <v>ধান</v>
       </c>
       <c r="D17" t="str">
-        <v>বস্তু</v>
+        <v>পাট</v>
       </c>
       <c r="E17" t="str">
-        <v>শিক্ষা</v>
+        <v>গোল আলু</v>
       </c>
       <c r="F17" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>নিচের কোনটি সবুজ সার জাতীয় ফসল?</v>
+        <v>নিচের কোনটি কৃষির তথ্য ও সেবা প্রাপ্তির প্রধান উৎস?</v>
       </c>
       <c r="B18" t="str">
-        <v>চিনা</v>
+        <v>অভিজ্ঞ কৃষক</v>
       </c>
       <c r="C18" t="str">
-        <v>কফি</v>
+        <v>কৃষক সভা</v>
       </c>
       <c r="D18" t="str">
-        <v>শনপাট</v>
+        <v>কৃষক বিদ্যালয়সমূহ</v>
       </c>
       <c r="E18" t="str">
-        <v>তিল</v>
+        <v>এনজিও</v>
       </c>
       <c r="F18" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>BARI-এর প্রধান কার্যালয় কোথায় ?</v>
+        <v>বাংলাদেশে কত প্রকার মসলার চাষ হয়?</v>
       </c>
       <c r="B19" t="str">
-        <v>গাজীপুর</v>
+        <v>১৪ প্রকার</v>
       </c>
       <c r="C19" t="str">
-        <v>ফরিদপুর</v>
+        <v>১৭ প্রকার</v>
       </c>
       <c r="D19" t="str">
-        <v>জামালপুর</v>
+        <v>৫০ প্রকার</v>
       </c>
       <c r="E19" t="str">
-        <v>পিরোজপুর</v>
+        <v>৭০ প্রকার</v>
       </c>
       <c r="F19" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BRRI এর প্রধান কার্যালয় কোথায় ?</v>
+        <v>স্থানীয় 'কৃষি তথ্য ভাণ্ডার' বলা হয় কাকে?</v>
       </c>
       <c r="B20" t="str">
-        <v>রাজশাহী</v>
+        <v>সাধারণ কৃষক</v>
       </c>
       <c r="C20" t="str">
-        <v>দিনাজপুর</v>
+        <v>অভিজ্ঞ কৃষক</v>
       </c>
       <c r="D20" t="str">
-        <v>ময়মনসিংহ</v>
+        <v>বয়স্ক কৃষক</v>
       </c>
       <c r="E20" t="str">
-        <v>গাজীপুর</v>
+        <v>কৃষক সভা</v>
       </c>
       <c r="F20" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>বাংলাদেশে কৃষি গবেষণা কাউন্সিল প্রতিষ্ঠিত হয় কত সালে?</v>
+        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
       </c>
       <c r="B21" t="str">
-        <v>১৯৭১ সালে</v>
+        <v>প্রতিটি গাছের আলাদাভাবে যত্ন নেওয়া হয়</v>
       </c>
       <c r="C21" t="str">
-        <v>১৯৭২ সালে</v>
+        <v>জমির সমস্ত ফসল ধাপে ধাপে পরিপক্ব ও সংগ্রহ করতে হয়</v>
       </c>
       <c r="D21" t="str">
-        <v>১৯৭৩ সালে</v>
+        <v>মৌসুমের শুরুতে দাম কম থাকে পরবর্তীতে দাম বাড়ে</v>
       </c>
       <c r="E21" t="str">
-        <v>১৯৭৪ সালে</v>
+        <v>তুলনামূলকভাবে বেশি যত্নের প্রয়োজন হয়</v>
       </c>
       <c r="F21" t="str">
         <v>C</v>
@@ -821,139 +821,139 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>‘এ টু আই' প্রকল্প সেবা কীসের মাধ্যমে দেওয়া হয়?</v>
+        <v>কৃষিতথ্য সার্ভিসের সদর দপ্তর কোথায় অবস্থিত?</v>
       </c>
       <c r="B22" t="str">
-        <v>এনজিও</v>
+        <v>জয়দেবপুর</v>
       </c>
       <c r="C22" t="str">
-        <v>ইন্টারনেট</v>
+        <v>মহাখালী</v>
       </c>
       <c r="D22" t="str">
-        <v>উঠন ঠৈকক</v>
+        <v>ধানমন্ডি</v>
       </c>
       <c r="E22" t="str">
-        <v>স্থানীয় প্রতিষ্ঠান</v>
+        <v>খামার বাড়ি</v>
       </c>
       <c r="F22" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>নিচের কোনটি মাঠ ফসল ?</v>
+        <v>শিল্প ফসল কোনটি?</v>
       </c>
       <c r="B23" t="str">
-        <v>গম</v>
+        <v>যব</v>
       </c>
       <c r="C23" t="str">
-        <v>আম</v>
+        <v>পাট</v>
       </c>
       <c r="D23" t="str">
-        <v>টমেটো</v>
+        <v>মাষকলাই</v>
       </c>
       <c r="E23" t="str">
-        <v>ফুলকপি</v>
+        <v>তাল</v>
       </c>
       <c r="F23" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>কৃষক সভার মূল উদ্দেশ্য কী?</v>
+        <v>টমেটোকে উদ্যান ফসল বলার কারণ-</v>
       </c>
       <c r="B24" t="str">
-        <v>কৃষি উৎপাদন বৃদ্ধি</v>
+        <v>সমস্ত ফসল একত্রে সংগ্রহ করা হয়</v>
       </c>
       <c r="C24" t="str">
-        <v>কৃষকদের সংখ্যা বৃদ্ধি</v>
+        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
       </c>
       <c r="D24" t="str">
-        <v>কৃষি জমির পরিমাণ বৃদ্ধি</v>
+        <v>নিচু ও মাঝারি নিচু জমিতে চাষ করা যায়</v>
       </c>
       <c r="E24" t="str">
-        <v>কৃষকদের অভিজ্ঞতা বৃদ্ধি</v>
+        <v>ফসলের দাম মৌসুমের শুরুতে কম থাকে</v>
       </c>
       <c r="F24" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>নিচের কোন প্রতিষ্ঠানটি শুধুমাত্র ধান নিয়ে গবেষণা করে?</v>
+        <v>বাউকুলের উদ্ভাবক প্রতিষ্ঠান কোনটি?</v>
       </c>
       <c r="B25" t="str">
-        <v>BARI</v>
+        <v>বা.কৃ.বি.</v>
       </c>
       <c r="C25" t="str">
-        <v>BINA</v>
+        <v>শে.কৃ.বি.</v>
       </c>
       <c r="D25" t="str">
-        <v>BADC</v>
+        <v>বারি</v>
       </c>
       <c r="E25" t="str">
-        <v>BRRI</v>
+        <v>বিজেআরআই</v>
       </c>
       <c r="F25" t="str">
-        <v>D</v>
+        <v>A</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>স্থানীয় 'কৃষি তথ্য ভাণ্ডার' বলা হয় কাকে?</v>
+        <v>দেশের একমাত্র ফিসারিজ কলেজটি কোন জেলায় অবস্থিত?</v>
       </c>
       <c r="B26" t="str">
-        <v>সাধারণ কৃষক</v>
+        <v>জামালপুর</v>
       </c>
       <c r="C26" t="str">
-        <v>অভিজ্ঞ কৃষক</v>
+        <v>ফরিদপুর</v>
       </c>
       <c r="D26" t="str">
-        <v>বয়স্ক কৃষক</v>
+        <v>যশোর</v>
       </c>
       <c r="E26" t="str">
-        <v>কৃষক সভা</v>
+        <v>রাজশাহী</v>
       </c>
       <c r="F26" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>উঠোন বৈঠকে কতজন কৃষক অংশগ্রহণ করে?</v>
+        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয় কত সালে প্রতিষ্ঠিত হয়?</v>
       </c>
       <c r="B27" t="str">
-        <v>৫-১০ জন</v>
+        <v>১৯৫৭</v>
       </c>
       <c r="C27" t="str">
-        <v>১০-১৫ জন</v>
+        <v>১৯৬১</v>
       </c>
       <c r="D27" t="str">
-        <v>১৫-২০ জন</v>
+        <v>১৯৬৫</v>
       </c>
       <c r="E27" t="str">
-        <v>২৫-৩০ জন</v>
+        <v>১৯৬৯</v>
       </c>
       <c r="F27" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>কতভাগ জমিতে উদ্যান ফসলের চাষ হয়?</v>
+        <v>বাংলাদেশে উৎপাদিত দানা ফসলের কত ভাগ ধান থেকে আসে?</v>
       </c>
       <c r="B28" t="str">
-        <v>৭০ ভাগ</v>
+        <v>৬০-৬৫%</v>
       </c>
       <c r="C28" t="str">
-        <v>৫০ ভাগ</v>
+        <v>৭০-৭৫%</v>
       </c>
       <c r="D28" t="str">
-        <v>৩০ ভাগ</v>
+        <v>৭৮-৮০%</v>
       </c>
       <c r="E28" t="str">
-        <v>১৪ ভাগ</v>
+        <v>৯০-৯৫%</v>
       </c>
       <c r="F28" t="str">
         <v>C</v>
@@ -961,139 +961,139 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>নিচের কোন ফসলটি ধাপে ধাপে সংগ্রহ করা হয়? .</v>
+        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
       </c>
       <c r="B29" t="str">
-        <v>পিয়াজ</v>
+        <v>ধাপে ধাপে পরিপক্ক হয়</v>
       </c>
       <c r="C29" t="str">
-        <v>আদা</v>
+        <v>শুকিয়ে ব্যবহার করা হয়</v>
       </c>
       <c r="D29" t="str">
-        <v>শিষ</v>
+        <v>বেড়া দেওয়া প্রয়োজন</v>
       </c>
       <c r="E29" t="str">
-        <v>আলু</v>
+        <v>বেশি যত্নের প্রয়োজন</v>
       </c>
       <c r="F29" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>নিচের কোনটি কৃষির তথ্য ও সেবা প্রাপ্তির প্রধান উৎস?</v>
+        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয় কত সালে প্রতিষ্ঠিত হয় ?</v>
       </c>
       <c r="B30" t="str">
-        <v>অভিজ্ঞ কৃষক</v>
+        <v>১৯৫৭</v>
       </c>
       <c r="C30" t="str">
-        <v>কৃষক সভা</v>
+        <v>১৯৬১</v>
       </c>
       <c r="D30" t="str">
-        <v>কৃষক বিদ্যালয়সমূহ</v>
+        <v>১৯৬৫</v>
       </c>
       <c r="E30" t="str">
-        <v>এনজিও</v>
+        <v>১৯৬৯</v>
       </c>
       <c r="F30" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>নিচের কোন প্রতিষ্ঠানটি তৈলবীজ নিয়ে গবেষণা করে?</v>
+        <v>BARI-এর প্রধান কার্যালয় কোথায় ?</v>
       </c>
       <c r="B31" t="str">
-        <v>BSRI</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="C31" t="str">
-        <v>BINA</v>
+        <v>ফরিদপুর</v>
       </c>
       <c r="D31" t="str">
-        <v>BTRI</v>
+        <v>জামালপুর</v>
       </c>
       <c r="E31" t="str">
-        <v>BARI</v>
+        <v>পিরোজপুর</v>
       </c>
       <c r="F31" t="str">
-        <v>D</v>
+        <v>A</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>BRRI এর প্রধান কার্যালয় কোথায়?</v>
+        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট এর আঞ্চলিক কার্যালয় কয়টি?</v>
       </c>
       <c r="B32" t="str">
-        <v>রাজশাহী</v>
+        <v>৩টি</v>
       </c>
       <c r="C32" t="str">
-        <v>দিনাজপুর</v>
+        <v>৫টি</v>
       </c>
       <c r="D32" t="str">
-        <v>ময়মনসিংহ</v>
+        <v>৬টি</v>
       </c>
       <c r="E32" t="str">
-        <v>গাজীপুর</v>
+        <v>৮টি</v>
       </c>
       <c r="F32" t="str">
-        <v>D</v>
+        <v>C</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>হাজী মোহাম্মদ দানেশ বিজ্ঞান ও প্রযুক্তি বিশ্ববিদ্যালয় কোন জেলায় অবস্থিত?</v>
+        <v>কোনটি মশলা জাতীয় ফসল?</v>
       </c>
       <c r="B33" t="str">
-        <v>গাজীপুর</v>
+        <v>পিয়াজ</v>
       </c>
       <c r="C33" t="str">
-        <v>দিনাজপুর</v>
+        <v>আলু</v>
       </c>
       <c r="D33" t="str">
-        <v>ময়মনসিংহ</v>
+        <v>শসা</v>
       </c>
       <c r="E33" t="str">
-        <v>রাজশাহী</v>
+        <v>ফুলকপি</v>
       </c>
       <c r="F33" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>কৃষক সভায় কতজন কৃষক অংশগ্রহণ করেন?</v>
+        <v>ফসলের নতুন নতুন জাত উদ্ভাবন ও উন্নয়ন সাধনের কাজ করে নিচের কোন প্রতিষ্ঠানটি?</v>
       </c>
       <c r="B34" t="str">
-        <v>১০-২০ জন</v>
+        <v>BARI</v>
       </c>
       <c r="C34" t="str">
-        <v>৩০-৪০ জন</v>
+        <v>BINA</v>
       </c>
       <c r="D34" t="str">
-        <v>৫০-৬০ জন</v>
+        <v>BARC</v>
       </c>
       <c r="E34" t="str">
-        <v>৭০-৮০ জন</v>
+        <v>BRRI</v>
       </c>
       <c r="F34" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>BARI-এর প্রধান কার্যালয় কোথায়?</v>
+        <v>আমাদের দেশে কৃষির আওতায় কত ধরনের ফসল চাষ করা হয়?</v>
       </c>
       <c r="B35" t="str">
-        <v>গাজীপুর</v>
+        <v>প্রায় ১২৪ ধরনের</v>
       </c>
       <c r="C35" t="str">
-        <v>জামালপুর</v>
+        <v>প্রায় ২২৪ ধরনের</v>
       </c>
       <c r="D35" t="str">
-        <v>ফরিদপুর</v>
+        <v>প্রায় ৩২৪ ধরনের</v>
       </c>
       <c r="E35" t="str">
-        <v>পিরোজপুর</v>
+        <v>প্রায় ৪২৪ ধরনের</v>
       </c>
       <c r="F35" t="str">
         <v>A</v>
@@ -1101,79 +1101,79 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>নিচের কোনটি কৃষি সম্প্রসারণ অধিদপ্তরের ওয়েবসাইট।</v>
+        <v>কৃষি তথ্যের জন্য মোবাইল ফোনের জিজ্ঞাসা নাম্বার কোনটি?</v>
       </c>
       <c r="B36" t="str">
-        <v>www.ais.gov.bd</v>
+        <v>১২১০</v>
       </c>
       <c r="C36" t="str">
-        <v>www.dae.gov.bd</v>
+        <v>৭৮৬৮</v>
       </c>
       <c r="D36" t="str">
-        <v>www.moa.gov.bd</v>
+        <v>৭৬৭৬</v>
       </c>
       <c r="E36" t="str">
-        <v>www.brri.gov.bd</v>
+        <v>৭৮৭৮</v>
       </c>
       <c r="F36" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>নিচের কোনটি দানাজাতীয় ফসল?</v>
+        <v>নিচের কোন প্রতিষ্ঠান কৃষক সভার আয়োজন করে?</v>
       </c>
       <c r="B37" t="str">
-        <v>মসুর</v>
+        <v>কৃষি সম্প্রসারণ অধিদপ্তর</v>
       </c>
       <c r="C37" t="str">
-        <v>সরিষা</v>
+        <v>বাংলাদেশ কৃষি উন্নয়ন কর্পোরেশন</v>
       </c>
       <c r="D37" t="str">
-        <v>ভুট্টা</v>
+        <v>বাংলাদেশ কৃষি গবেষণা কাউন্সিল</v>
       </c>
       <c r="E37" t="str">
-        <v>ছোলা</v>
+        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট</v>
       </c>
       <c r="F37" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ফসলের নতুন নতুন জাত উদ্ভাবন ও উন্নয়ন সাধনের কাজ করে নিচের কোন প্রতিষ্ঠানটি?</v>
+        <v>নিচের কোনটি সবুজ সার জাতীয় ফসল?</v>
       </c>
       <c r="B38" t="str">
-        <v>BARI</v>
+        <v>চিনা</v>
       </c>
       <c r="C38" t="str">
-        <v>BINA</v>
+        <v>কফি</v>
       </c>
       <c r="D38" t="str">
-        <v>BARC</v>
+        <v>শনপাট</v>
       </c>
       <c r="E38" t="str">
-        <v>BRRI</v>
+        <v>তিল</v>
       </c>
       <c r="F38" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>বাংলাদেশে উৎপাদিত দানা ফসলের কত ভাগ ধান থেকে আসে?</v>
+        <v>নিচের কোনটি দানাজাতীয় ফসল?</v>
       </c>
       <c r="B39" t="str">
-        <v>৬০-৬৫%</v>
+        <v>মসুর</v>
       </c>
       <c r="C39" t="str">
-        <v>৭০-৭৫%</v>
+        <v>সরিষা</v>
       </c>
       <c r="D39" t="str">
-        <v>৭৮-৮০%</v>
+        <v>ভুট্টা</v>
       </c>
       <c r="E39" t="str">
-        <v>৯০-৯৫%</v>
+        <v>ছোলা</v>
       </c>
       <c r="F39" t="str">
         <v>C</v>
@@ -1181,19 +1181,19 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
+        <v>পাটকে মাঠ ফসল বলার কারণ—</v>
       </c>
       <c r="B40" t="str">
-        <v>প্রতিটি গাছের আলাদাভাবে যত্ন নেওয়া হয়</v>
+        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
       </c>
       <c r="C40" t="str">
-        <v>জমির সমস্ত ফসল ধাপে ধাপে পরিপক্ক ও সংগ্রহ করতে হয়</v>
+        <v>ফসলের লাভ ও ব্যয়ের অনুপাত বেশি হয়</v>
       </c>
       <c r="D40" t="str">
-        <v>মৌসুমের শুরুতে দাম কম থাকে পরবর্তীতে দাম বাড়ে</v>
+        <v>সমস্ত ফসল একত্রে পরিপক্ক ও সংগ্রহ করা হয়</v>
       </c>
       <c r="E40" t="str">
-        <v>তুলনামূলকভাবে বেশি যত্নের প্রয়োজন হয়।</v>
+        <v>ফসলের মূল্য মৌসুমের শুরুতে বেশি হয়</v>
       </c>
       <c r="F40" t="str">
         <v>C</v>
@@ -1201,39 +1201,39 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>মিঠা পানিতে কত প্রজাতির মাছ রয়েছে?</v>
+        <v>কোনটি কনড্রিকথিস শ্রেণির মাছ?</v>
       </c>
       <c r="B41" t="str">
-        <v>২৪০</v>
+        <v>কাতলা</v>
       </c>
       <c r="C41" t="str">
-        <v>২৫০</v>
+        <v>হাঙ্গর</v>
       </c>
       <c r="D41" t="str">
-        <v>২৬০</v>
+        <v>তেলাপিয়া</v>
       </c>
       <c r="E41" t="str">
-        <v>৪৭৫</v>
+        <v>কৈ</v>
       </c>
       <c r="F41" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>শিল্প ফসল কোনটি?</v>
+        <v>বিদেশি অর্থায়নে কৃষি উন্নয়নের লক্ষ্যে কৃষি তথ্য সরবরাহ করে কোন প্রতিষ্ঠান?</v>
       </c>
       <c r="B42" t="str">
-        <v>যব</v>
+        <v>ASA</v>
       </c>
       <c r="C42" t="str">
-        <v>পাট</v>
+        <v>JIСА</v>
       </c>
       <c r="D42" t="str">
-        <v>মাষকলাই</v>
+        <v>CARE</v>
       </c>
       <c r="E42" t="str">
-        <v>তাল</v>
+        <v>TMSS</v>
       </c>
       <c r="F42" t="str">
         <v>B</v>
@@ -1241,199 +1241,199 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>দেশের সবচেয়ে বড় শিক্ষা প্রতিষ্ঠান কোনটি?</v>
+        <v>মাছ কোন পর্বের অন্তর্গত?</v>
       </c>
       <c r="B43" t="str">
-        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয়</v>
+        <v>আর্থ্রোপোডা</v>
       </c>
       <c r="C43" t="str">
-        <v>ঢাকা বিশ্ববিদ্যালয়</v>
+        <v>কর্ডাটা</v>
       </c>
       <c r="D43" t="str">
-        <v>শেরে বাংলা কৃষি বিশ্ববিদ্যালয়</v>
+        <v>অ্যানিলিডা</v>
       </c>
       <c r="E43" t="str">
-        <v>রাজশাহী বিশ্ববিদ্যালয়</v>
+        <v>পরিফেরা</v>
       </c>
       <c r="F43" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>কৃষির ক্ষেত্র কতটি?</v>
+        <v>উঠোন বৈঠকের উদ্দেশ্য-</v>
       </c>
       <c r="B44" t="str">
-        <v>৩</v>
+        <v>অন্যায় থেকে বিরত রাখা</v>
       </c>
       <c r="C44" t="str">
-        <v>৪</v>
+        <v>কৃষি তথ্য প্রচার করা</v>
       </c>
       <c r="D44" t="str">
-        <v>৫</v>
+        <v>স্কুলে যেতে উৎসাহ প্রদান</v>
       </c>
       <c r="E44" t="str">
-        <v>৬</v>
+        <v>সবজির পুষ্টিগুণ প্রচার</v>
       </c>
       <c r="F44" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয় কত সালে প্রতিষ্ঠিত হয়?</v>
+        <v>১ উদ্যান ফসল একে একে উত্তোলন করা হয় কেন?</v>
       </c>
       <c r="B45" t="str">
-        <v>১৯৫৭</v>
+        <v>শ্রমিকের অপ্রতুলতা</v>
       </c>
       <c r="C45" t="str">
-        <v>১৯৬১</v>
+        <v>প্রক্রিয়াজাতকরণের অভাবে</v>
       </c>
       <c r="D45" t="str">
-        <v>১৯৬৫</v>
+        <v>বাজারমূল্য কমে যায় বলে</v>
       </c>
       <c r="E45" t="str">
-        <v>১৯৬৯</v>
+        <v>ধাপে ধাপে পরিপক্ক হয় বলে</v>
       </c>
       <c r="F45" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>নিচের কোনটি মাঠ ফসল?</v>
+        <v>নিচের কোন ফসলটি ধাপে ধাপে সংগ্রহ করা হয়? .</v>
       </c>
       <c r="B46" t="str">
-        <v>আম</v>
+        <v>পিয়াজ</v>
       </c>
       <c r="C46" t="str">
-        <v>সরিষা</v>
+        <v>আদা</v>
       </c>
       <c r="D46" t="str">
-        <v>ফুলকপি</v>
+        <v>শিষ</v>
       </c>
       <c r="E46" t="str">
-        <v>পালংশাক</v>
+        <v>আলু</v>
       </c>
       <c r="F46" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>নতুন নতুন প্রযুক্তি সম্পর্কে খোজ খবর রাখেন কে?</v>
+        <v>টমেটোকে উদ্যান ফসল বলার কারণ—</v>
       </c>
       <c r="B47" t="str">
-        <v>অভিজ্ঞ কৃষক</v>
+        <v>সমস্ত ফসল একত্রে সংগ্রহ করা হয়</v>
       </c>
       <c r="C47" t="str">
-        <v>বয়স্ক কৃষক</v>
+        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
       </c>
       <c r="D47" t="str">
-        <v>স্থানীয় মেম্বার</v>
+        <v>নিচু ও মাঝারি নিচু জমিতে চাষ করা যায়</v>
       </c>
       <c r="E47" t="str">
-        <v>স্কুল শিক্ষক</v>
+        <v>ফসলের দাম মৌসুমের শুরুতে কম থাকে</v>
       </c>
       <c r="F47" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>কৃষির কোন ক্ষেত্রটি সরাসরি পরিবেশ রক্ষায় গুরুত্বপূর্ণ ভূমিকা পালন করে?</v>
+        <v>শিল্প ফসল কোনটি?</v>
       </c>
       <c r="B48" t="str">
-        <v>গবাদিপশু</v>
+        <v>গম</v>
       </c>
       <c r="C48" t="str">
-        <v>পোলট্রি</v>
+        <v>রাবার</v>
       </c>
       <c r="D48" t="str">
-        <v>মৎস্য</v>
+        <v>বাসক</v>
       </c>
       <c r="E48" t="str">
-        <v>সামাজিক বনায়ন</v>
+        <v>নেপিয়ার</v>
       </c>
       <c r="F48" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>আমাদের দেশে কৃষির আওতায় কত ধরনের ফসল চাষ করা হয়?</v>
+        <v>প্রাণিজগতকে কয়টি পর্বে ভাগ করা যায়?</v>
       </c>
       <c r="B49" t="str">
-        <v>প্রায় ১২৪ ধরনের</v>
+        <v>৮টি</v>
       </c>
       <c r="C49" t="str">
-        <v>প্রায় ২২৪ ধরনের</v>
+        <v>৯টি</v>
       </c>
       <c r="D49" t="str">
-        <v>প্রায় ৩২৪ ধরনের</v>
+        <v>১০টি</v>
       </c>
       <c r="E49" t="str">
-        <v>প্রায় ৪২৪ ধরনের</v>
+        <v>১১টি</v>
       </c>
       <c r="F49" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>বাংলাদেশ পাট গবেষণা ইনস্টিটিউট কোথায় অবস্থিত?</v>
+        <v>কৃষক সভার প্রয়োজন কেন?</v>
       </c>
       <c r="B50" t="str">
-        <v>ঢাকা</v>
+        <v>কৃষি উপকরণ সরবরাহ</v>
       </c>
       <c r="C50" t="str">
-        <v>গাজীপুর</v>
+        <v>কুশল বিনিময়</v>
       </c>
       <c r="D50" t="str">
-        <v>টাঙ্গাইল</v>
+        <v>কৃষি ঋণ গ্রহণ</v>
       </c>
       <c r="E50" t="str">
-        <v>পাবনা</v>
+        <v>কৃষি তথ্য আদান-প্রদান</v>
       </c>
       <c r="F50" t="str">
-        <v>A</v>
+        <v>D</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>শিল্প ফসল কোনটি?</v>
+        <v>দেশের সবচেয়ে বড় শিক্ষা প্রতিষ্ঠান কোনটি?</v>
       </c>
       <c r="B51" t="str">
-        <v>গম</v>
+        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয়</v>
       </c>
       <c r="C51" t="str">
-        <v>রাবার</v>
+        <v>ঢাকা বিশ্ববিদ্যালয়</v>
       </c>
       <c r="D51" t="str">
-        <v>বাসক</v>
+        <v>শেরে বাংলা কৃষি বিশ্ববিদ্যালয়</v>
       </c>
       <c r="E51" t="str">
-        <v>নেপিয়ার</v>
+        <v>রাজশাহী বিশ্ববিদ্যালয়</v>
       </c>
       <c r="F51" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
+        <v>BARI কোথায় অবস্থিত?</v>
       </c>
       <c r="B52" t="str">
-        <v>ধাপে ধাপে পরিপক্ক হয়</v>
+        <v>ময়মনসিংহ</v>
       </c>
       <c r="C52" t="str">
-        <v>শুকিয়ে ব্যবহার করা হয়</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="D52" t="str">
-        <v>বেড়া দেওয়া প্রয়োজন</v>
+        <v>সাভার</v>
       </c>
       <c r="E52" t="str">
-        <v>বেশি যত্নের প্রয়োজন</v>
+        <v>সিলেট</v>
       </c>
       <c r="F52" t="str">
         <v>B</v>
@@ -1441,239 +1441,239 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>কৃষক সভার প্রয়োজন কেন?</v>
+        <v>পোল্ট্রি কোনটি?</v>
       </c>
       <c r="B53" t="str">
-        <v>কৃষি উপকরণ সরবরাহ</v>
+        <v>টিয়া</v>
       </c>
       <c r="C53" t="str">
-        <v>কুশল বিনিময়</v>
+        <v>টার্কি</v>
       </c>
       <c r="D53" t="str">
-        <v>কৃষি ঋণ গ্রহণ</v>
+        <v>ময়না</v>
       </c>
       <c r="E53" t="str">
-        <v>কৃষি তথ্য আদান-প্রদান</v>
+        <v>ঘুঘু</v>
       </c>
       <c r="F53" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>বাংলাদেশে কত প্রকার মসলার চাষ হয়?</v>
+        <v>কৃষির কোন ক্ষেত্রটি সরাসরি পরিবেশ রক্ষায় গুরুত্বপূর্ণ ভূমিকা পালন করে?</v>
       </c>
       <c r="B54" t="str">
-        <v>১৪ প্রকার</v>
+        <v>গবাদিপশু</v>
       </c>
       <c r="C54" t="str">
-        <v>১৭ প্রকার</v>
+        <v>পোলট্রি</v>
       </c>
       <c r="D54" t="str">
-        <v>৫০ প্রকার</v>
+        <v>মৎস্য</v>
       </c>
       <c r="E54" t="str">
-        <v>৭০ প্রকার</v>
+        <v>সামাজিক বনায়ন</v>
       </c>
       <c r="F54" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>চাষাবাদে যন্ত্রশক্তির ব্যবহার কত?</v>
+        <v>সর্বাধিক সংখ্যক কৃষি উপকরণ সরবরাহকারী প্রতিষ্ঠান কোনটি?</v>
       </c>
       <c r="B55" t="str">
-        <v>৪০%</v>
+        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয়</v>
       </c>
       <c r="C55" t="str">
-        <v>৫০%</v>
+        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট</v>
       </c>
       <c r="D55" t="str">
-        <v>৬০%</v>
+        <v>বাংলাদেশ ধান গবেষণা ইনস্টিটিউট</v>
       </c>
       <c r="E55" t="str">
-        <v>৮০%</v>
+        <v>বাংলাদেশ কৃষি উন্নয়ন কর্পোরেশন (BADC)</v>
       </c>
       <c r="F55" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>বাংলাদেশে প্রাণিজ আমিষের প্রায় কত ভাগ আসে মাছ থেকে?</v>
+        <v>কৃষি তথ্য সার্ভিসের সদর দপ্তর কোথায় অবস্থিত?</v>
       </c>
       <c r="B56" t="str">
-        <v>৪০%</v>
+        <v>জয়দেবপুর</v>
       </c>
       <c r="C56" t="str">
-        <v>৫০%</v>
+        <v>মহাখাল</v>
       </c>
       <c r="D56" t="str">
-        <v>৬০%</v>
+        <v>ধানমণ্ডি</v>
       </c>
       <c r="E56" t="str">
-        <v>৭০%</v>
+        <v>খামারবাড়ী</v>
       </c>
       <c r="F56" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>কৃষি তথ্য সংস্থা আত্মপ্রকাশ করে কত সালে?</v>
+        <v>বাংলাদেশ ধান গবেষণা ইনস্টিটিউট কোথায় অবস্থিত?</v>
       </c>
       <c r="B57" t="str">
-        <v>১৯৫০</v>
+        <v>ঢাকা</v>
       </c>
       <c r="C57" t="str">
-        <v>১৯৫৬</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="D57" t="str">
-        <v>১৯৬১</v>
+        <v>দিনাজপুর</v>
       </c>
       <c r="E57" t="str">
-        <v>১৯৬৫</v>
+        <v>পঞ্চগড়</v>
       </c>
       <c r="F57" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>কোনটি মশলা জাতীয় ফসল?</v>
+        <v>পাটকে মাঠ ফসল বলা কারণ-</v>
       </c>
       <c r="B58" t="str">
-        <v>পিয়াজ</v>
+        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
       </c>
       <c r="C58" t="str">
-        <v>আলু</v>
+        <v>ফসলের লাভ ও ব্যয়ের অনুপাত বেশি হয়</v>
       </c>
       <c r="D58" t="str">
-        <v>শসা</v>
+        <v>সমস্ত ফসল একত্রে পরিপক্ক ও সংগ্রহ করা হয়</v>
       </c>
       <c r="E58" t="str">
-        <v>ফুলকপি</v>
+        <v>ফসলের মূল্য মৌসুমের শুরুতে বেশি হয়</v>
       </c>
       <c r="F58" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>১ উদ্যান ফসল একে একে উত্তোলন করা হয় কেন?</v>
+        <v>নিচের কোনটি দানাজাতীয় ফসল?</v>
       </c>
       <c r="B59" t="str">
-        <v>শ্রমিকের অপ্রতুলতা</v>
+        <v>সূর্যমুখী</v>
       </c>
       <c r="C59" t="str">
-        <v>প্রক্রিয়াজাতকরণের অভাবে</v>
+        <v>কাউন</v>
       </c>
       <c r="D59" t="str">
-        <v>বাজারমূল্য কমে যায় বলে</v>
+        <v>শণপাট</v>
       </c>
       <c r="E59" t="str">
-        <v>ধাপে ধাপে পরিপক্ক হয় বলে</v>
+        <v>মেস্তা</v>
       </c>
       <c r="F59" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>নিচের কোনটি উদ্যান ফসল ?</v>
+        <v>মিঠা পানিতে কত প্রজাতির মাছ রয়েছে?</v>
       </c>
       <c r="B60" t="str">
-        <v>তুলা</v>
+        <v>২৪০</v>
       </c>
       <c r="C60" t="str">
-        <v>&lt;p&gt;ধান&lt;/p&gt;</v>
+        <v>২৫০</v>
       </c>
       <c r="D60" t="str">
-        <v>&lt;p&gt;পাট&lt;/p&gt;</v>
+        <v>২৬০</v>
       </c>
       <c r="E60" t="str">
-        <v>&lt;p&gt;গোল আলু&lt;/p&gt;</v>
+        <v>৪৭৫</v>
       </c>
       <c r="F60" t="str">
-        <v>D</v>
+        <v>C</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>কৃষি তথ্যের জন্য মোবাইল ফোনের জিজ্ঞাসা নাম্বার কোনটি?</v>
+        <v>ধানের জাত উদ্ভাবনকারী প্রতিষ্ঠান হচ্ছে-</v>
       </c>
       <c r="B61" t="str">
-        <v>১২১০</v>
+        <v>BARI</v>
       </c>
       <c r="C61" t="str">
-        <v>৭৮৬৮</v>
+        <v>BRRI</v>
       </c>
       <c r="D61" t="str">
-        <v>৭৬৭৬</v>
+        <v>BSRI</v>
       </c>
       <c r="E61" t="str">
-        <v>৭৮৭৮</v>
+        <v>SRDI</v>
       </c>
       <c r="F61" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>বিদেশি অর্থায়নে কৃষি উন্নয়নের লক্ষ্যে কৃষি তথ্য সরবরাহ করে কোন প্রতিষ্ঠান?</v>
+        <v>নিচের কোনটি স্বাদু পানির মাছ?</v>
       </c>
       <c r="B62" t="str">
-        <v>ASA</v>
+        <v>রুপচান্দা</v>
       </c>
       <c r="C62" t="str">
-        <v>JIСА</v>
+        <v>ছুরি</v>
       </c>
       <c r="D62" t="str">
-        <v>CARE</v>
+        <v>পোয়া</v>
       </c>
       <c r="E62" t="str">
-        <v>TMSS</v>
+        <v>মাগুর</v>
       </c>
       <c r="F62" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>কোন উৎস থেকে কৃষক কৃষি বিষয়ক সকল তথ্য পেতে পারে?</v>
+        <v>কৃষি শিক্ষক দুটি বিষয় নিয়ে বেশি আলোচনার কারণ কোনটি?</v>
       </c>
       <c r="B63" t="str">
-        <v>উঠোন বৈঠক</v>
+        <v>প্রধান খাদ্য</v>
       </c>
       <c r="C63" t="str">
-        <v>কৃষিশিক্ষা বই</v>
+        <v>অর্থনৈতিক গুরুত্ব</v>
       </c>
       <c r="D63" t="str">
-        <v>এনজিও</v>
+        <v>পুষ্টির চাহিদা পূরণ</v>
       </c>
       <c r="E63" t="str">
-        <v>ইউনিয়ন সেবাকেন্দ্র</v>
+        <v>উৎপাদন ঝুঁকি</v>
       </c>
       <c r="F63" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>নিচের কোনটি দানাজাতীয় ফসল?</v>
+        <v>বাংলাদেশে সর্বাধিক সংখ্যক উন্নত জাতের ধান উদ্ভাবক প্রতিষ্ঠান</v>
       </c>
       <c r="B64" t="str">
-        <v>সূর্যমুখী</v>
+        <v>BAU</v>
       </c>
       <c r="C64" t="str">
-        <v>কাউন</v>
+        <v>BRRI</v>
       </c>
       <c r="D64" t="str">
-        <v>শনপাট</v>
+        <v>BINA</v>
       </c>
       <c r="E64" t="str">
-        <v>মেস্তা</v>
+        <v>BARI</v>
       </c>
       <c r="F64" t="str">
         <v>B</v>
@@ -1681,139 +1681,139 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
+        <v>কৃষি বন কোন বনায়নের অন্তর্ভুক্ত?</v>
       </c>
       <c r="B65" t="str">
-        <v>প্রতিটি গাছের আলাদাভাবে যত্ন নেওয়া হয়</v>
+        <v>সামাজিক বন</v>
       </c>
       <c r="C65" t="str">
-        <v>জমির সমস্ত ফসল ধাপে ধাপে পরিপক্ব ও সংগ্রহ করতে হয়</v>
+        <v>সমতল বন</v>
       </c>
       <c r="D65" t="str">
-        <v>মৌসুমের শুরুতে দাম কম থাকে পরবর্তীতে দাম বাড়ে</v>
+        <v>পাহাড়ি বন</v>
       </c>
       <c r="E65" t="str">
-        <v>তুলনামূলকভাবে বেশি যত্নের প্রয়োজন হয়</v>
+        <v>ম্যানগ্রোভ বন</v>
       </c>
       <c r="F65" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>ধানের জাত উদ্ভাবনকারী প্রতিষ্ঠান হচ্ছে-</v>
+        <v>দেশের মোট আবাদি জমির শতকরা কত ভাগ মাঠ ফসল?</v>
       </c>
       <c r="B66" t="str">
-        <v>BARI</v>
+        <v>৩০ ভাগ</v>
       </c>
       <c r="C66" t="str">
-        <v>BRRI</v>
+        <v>৫০ ভাগ</v>
       </c>
       <c r="D66" t="str">
-        <v>BSRI</v>
+        <v>৭০ ভাগ</v>
       </c>
       <c r="E66" t="str">
-        <v>SRDI</v>
+        <v>৯০ ভাগ</v>
       </c>
       <c r="F66" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>নিচের কোনটি দানা জাতীয় ফসল?</v>
+        <v>‘এ টু আই' প্রকল্প সেবা কীসের মাধ্যমে দেওয়া হয়?</v>
       </c>
       <c r="B67" t="str">
-        <v>ছোলা</v>
+        <v>এনজিও</v>
       </c>
       <c r="C67" t="str">
-        <v>সরিষা</v>
+        <v>ইন্টারনেট</v>
       </c>
       <c r="D67" t="str">
-        <v>চীনা বাদাম</v>
+        <v>উঠন ঠৈকক</v>
       </c>
       <c r="E67" t="str">
-        <v>ধান</v>
+        <v>স্থানীয় প্রতিষ্ঠান</v>
       </c>
       <c r="F67" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>নিচের কোনটি দানাজাতীয় ফসল?</v>
+        <v>কৃষির ক্ষেত্র কতটি?</v>
       </c>
       <c r="B68" t="str">
-        <v>সূর্যমুখী</v>
+        <v>৩</v>
       </c>
       <c r="C68" t="str">
-        <v>কাউন</v>
+        <v>৪</v>
       </c>
       <c r="D68" t="str">
-        <v>শণপাট</v>
+        <v>৫</v>
       </c>
       <c r="E68" t="str">
-        <v>মেস্তা</v>
+        <v>৬</v>
       </c>
       <c r="F68" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>কোন প্রতিষ্ঠান কৃষকদের সার, বীজ কীটনাশক ও কৃষি যন্ত্রপাতি সরবরাহ করে?</v>
+        <v>বাংলাদেশ কৃষি গবেষণা প্রতিষ্ঠান কত সালে প্রতিষ্ঠিত হয়?</v>
       </c>
       <c r="B69" t="str">
-        <v>BADC</v>
+        <v>১৯৭৪ সালে</v>
       </c>
       <c r="C69" t="str">
-        <v>BFDC</v>
+        <v>১৯৭৬ সালে</v>
       </c>
       <c r="D69" t="str">
-        <v>BARI</v>
+        <v>১৯৭৮ সালে</v>
       </c>
       <c r="E69" t="str">
-        <v>BRRI</v>
+        <v>১৯৮০ সালে</v>
       </c>
       <c r="F69" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>হাতের স্পর্শের মাধ্যমে তথ্য প্রাপ্তির জন্য তৈরি করা হয়েছে কোনটি</v>
+        <v>উদ্যান ফসলগুলো সাধারণত কত ভাগে বিভক্ত?</v>
       </c>
       <c r="B70" t="str">
-        <v>কিয়স্ক</v>
+        <v>২ ভাগে</v>
       </c>
       <c r="C70" t="str">
-        <v>কিমানো</v>
+        <v>৩ ভাগে</v>
       </c>
       <c r="D70" t="str">
-        <v>এস্কিমো</v>
+        <v>৪ ভাগে</v>
       </c>
       <c r="E70" t="str">
-        <v>কিয়াটো</v>
+        <v>৫ ভাগে</v>
       </c>
       <c r="F70" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>গবেষণার জন্য বৈদেশিক সাহায্য আনয়নের ব্যবস্থা করে কোন প্রতিষ্ঠান?</v>
+        <v>দেশের একমাত্র ফিসারিজ কলেজটি কোন জেলায় অবস্থিত?</v>
       </c>
       <c r="B71" t="str">
-        <v>BARC</v>
+        <v>জামালপুর</v>
       </c>
       <c r="C71" t="str">
-        <v>BADC</v>
+        <v>ফরিদপুর</v>
       </c>
       <c r="D71" t="str">
-        <v>BARI</v>
+        <v>যশোর</v>
       </c>
       <c r="E71" t="str">
-        <v>BRRI</v>
+        <v>রাজশাহী</v>
       </c>
       <c r="F71" t="str">
         <v>A</v>
@@ -1821,159 +1821,159 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>কৃষিতথ্য সার্ভিসের সদর দপ্তর কোথায় অবস্থিত?</v>
+        <v>বাংলাদেশে প্রাণিজ আমিষের প্রায় কত ভাগ আসে মাছ থেকে?</v>
       </c>
       <c r="B72" t="str">
-        <v>জয়দেবপুর</v>
+        <v>৪০%</v>
       </c>
       <c r="C72" t="str">
-        <v>মহাখালী</v>
+        <v>৫০%</v>
       </c>
       <c r="D72" t="str">
-        <v>ধানমণ্ডি</v>
+        <v>৬০%</v>
       </c>
       <c r="E72" t="str">
-        <v>খামার বাড়ি</v>
+        <v>৭০%</v>
       </c>
       <c r="F72" t="str">
-        <v>D</v>
+        <v>C</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>দেশের মোট আবাদি জমির শতকরা কত ভাগ মাঠ ফসল?</v>
+        <v>নিচের কোনটি গবেষণা প্রতিষ্ঠান?</v>
       </c>
       <c r="B73" t="str">
-        <v>৩০ ভাগ</v>
+        <v>BADC</v>
       </c>
       <c r="C73" t="str">
-        <v>৫০ ভাগ</v>
+        <v>SRDI</v>
       </c>
       <c r="D73" t="str">
-        <v>৭০ ভাগ</v>
+        <v>BRAC</v>
       </c>
       <c r="E73" t="str">
-        <v>৯০ ভাগ</v>
+        <v>BAU</v>
       </c>
       <c r="F73" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>নিচের কোনটি কৃষি সম্প্রসারণ প্রতিষ্ঠান।</v>
+        <v>নিচের কোনটি কৃষি গবেষণা প্রতিষ্ঠান?</v>
       </c>
       <c r="B74" t="str">
-        <v>DAE</v>
+        <v>BAU</v>
       </c>
       <c r="C74" t="str">
+        <v>BADC</v>
+      </c>
+      <c r="D74" t="str">
         <v>BARI</v>
       </c>
-      <c r="D74" t="str">
-        <v>BRRI</v>
-      </c>
       <c r="E74" t="str">
-        <v>BINA</v>
+        <v>SAU</v>
       </c>
       <c r="F74" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>কৃষির ইংরেজিতে Agriculture শব্দটি এসেছে-</v>
+        <v>নিচের কোনটি মাঠ ফসল?</v>
       </c>
       <c r="B75" t="str">
-        <v>ল্যাটিন শব্দ হতে</v>
+        <v>আম</v>
       </c>
       <c r="C75" t="str">
-        <v>ব্রিটিশ শব্দ হতে</v>
+        <v>সরিষা</v>
       </c>
       <c r="D75" t="str">
-        <v>ফারসি শব্দ হতে</v>
+        <v>ফুলকপি</v>
       </c>
       <c r="E75" t="str">
-        <v>চৈনিক শব্দ হতে</v>
+        <v>পালংশাক</v>
       </c>
       <c r="F75" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>নিচের কোনটি গবেষণা প্রতিষ্ঠান?</v>
+        <v>প্রাণিজ আমিষের প্রায় কত ভাগ মাছ থেকে আসে?</v>
       </c>
       <c r="B76" t="str">
-        <v>BADC</v>
+        <v>৪০%</v>
       </c>
       <c r="C76" t="str">
-        <v>SRDI</v>
+        <v>৫০%</v>
       </c>
       <c r="D76" t="str">
-        <v>BRAC</v>
+        <v>৬০%</v>
       </c>
       <c r="E76" t="str">
-        <v>BAU</v>
+        <v>৭০%</v>
       </c>
       <c r="F76" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>একটি কৃষক সভায় অংশগ্রহণকারী সদস্যের সংখ্যা সাধারণত কত?</v>
+        <v>নিচের কোনটি মাঠ ফসল ?</v>
       </c>
       <c r="B77" t="str">
-        <v>২০-৩০ জন</v>
+        <v>গম</v>
       </c>
       <c r="C77" t="str">
-        <v>২৫-৩০ জন</v>
+        <v>আম</v>
       </c>
       <c r="D77" t="str">
-        <v>৩০-৪০ জন</v>
+        <v>টমেটো</v>
       </c>
       <c r="E77" t="str">
-        <v>৫০-৬০ জন</v>
+        <v>ফুলকপি</v>
       </c>
       <c r="F77" t="str">
-        <v>D</v>
+        <v>A</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>দেশের একমাত্র ফিসারিজ কলেজটি কোন জেলায় অবস্থিত?</v>
+        <v>উঠোন বৈঠকে কতজন কৃষক অংশগ্রহণ করে?</v>
       </c>
       <c r="B78" t="str">
-        <v>জামালপুর</v>
+        <v>৫-১০ জন</v>
       </c>
       <c r="C78" t="str">
-        <v>ফরিদপুর</v>
+        <v>১০-১৫ জন</v>
       </c>
       <c r="D78" t="str">
-        <v>যশোর</v>
+        <v>১৫-২০ জন</v>
       </c>
       <c r="E78" t="str">
-        <v>রাজশাহী</v>
+        <v>২৫-৩০ জন</v>
       </c>
       <c r="F78" t="str">
-        <v>A</v>
+        <v>D</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>একজন কৃষক কোন উৎস থেকে সবচেয়ে সহজ উপায়ে কৃষি সেবা পেতে পারে।</v>
+        <v>নিচের কোন প্রতিষ্ঠান কৃষক সভার আয়োজন করে?</v>
       </c>
       <c r="B79" t="str">
-        <v>ইন্টারনেট</v>
+        <v>কৃষি সম্প্রসারণ অধিদপ্তর</v>
       </c>
       <c r="C79" t="str">
-        <v>অভিজ্ঞ কৃষক</v>
+        <v>বাংলাদেশ কৃষি উন্নয়ন কর্পোরেশন</v>
       </c>
       <c r="D79" t="str">
-        <v>উঠোন বৈঠক</v>
+        <v>বাংলাদেশ কৃষি গবেষণা কাউন্সিল</v>
       </c>
       <c r="E79" t="str">
-        <v>কৃষিতথ্য সার্ভিস</v>
+        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট</v>
       </c>
       <c r="F79" t="str">
         <v>A</v>
@@ -1981,19 +1981,19 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>কৃষি তথ্যের সবচেয়ে বড় ভাণ্ডার কোনটি?</v>
+        <v>নিচের কোন প্রতিষ্ঠানটি তৈলবীজ নিয়ে গবেষণা করে?</v>
       </c>
       <c r="B80" t="str">
-        <v>কৃষি কথা পত্রিকা</v>
+        <v>BSRI</v>
       </c>
       <c r="C80" t="str">
-        <v>মোবাইল ফোন</v>
+        <v>BINA</v>
       </c>
       <c r="D80" t="str">
-        <v>টেলিভিশন</v>
+        <v>BTRI</v>
       </c>
       <c r="E80" t="str">
-        <v>ইন্টারনেট</v>
+        <v>BARI</v>
       </c>
       <c r="F80" t="str">
         <v>D</v>
@@ -2001,19 +2001,19 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>দেশের একমাত্র ফিসারিজ কলেজটি কোন জেলায় অবস্থিত?</v>
+        <v>একজন কৃষক কোন উৎস থেকে সবচেয়ে সহজ উপায়ে কৃষি সেবা পেতে পারে।</v>
       </c>
       <c r="B81" t="str">
-        <v>জামালপুর</v>
+        <v>ইন্টারনেট</v>
       </c>
       <c r="C81" t="str">
-        <v>ফরিদপুর</v>
+        <v>অভিজ্ঞ কৃষক</v>
       </c>
       <c r="D81" t="str">
-        <v>যশোর</v>
+        <v>উঠোন বৈঠক</v>
       </c>
       <c r="E81" t="str">
-        <v>রাজশাহী</v>
+        <v>কৃষিতথ্য সার্ভিস</v>
       </c>
       <c r="F81" t="str">
         <v>A</v>
@@ -2021,39 +2021,39 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>মাছ কোন পর্বের অন্তর্গত?</v>
+        <v>কৃষক সভার মূল উদ্দেশ্য কী?</v>
       </c>
       <c r="B82" t="str">
-        <v>আর্থ্রোপোডা</v>
+        <v>কৃষি উৎপাদন বৃদ্ধি</v>
       </c>
       <c r="C82" t="str">
-        <v>কর্ডাটা</v>
+        <v>কৃষকদের সংখ্যা বৃদ্ধি</v>
       </c>
       <c r="D82" t="str">
-        <v>অ্যানিলিডা</v>
+        <v>কৃষি জমির পরিমাণ বৃদ্ধি</v>
       </c>
       <c r="E82" t="str">
-        <v>পরিফেরা</v>
+        <v>কৃষকদের অভিজ্ঞতা বৃদ্ধি</v>
       </c>
       <c r="F82" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>আন্তর্জাতিক ধান গবেষণা প্রতিষ্ঠানের সাথে মিল রয়েছে এমন একটি প্রতিষ্ঠান বাংলাদেশে আছে সেটির নাম কী?</v>
+        <v>নদীর প্রবাহ বাধাপ্রাপ্ত হয়ে উৎপন্ন জলাশয়কে কি বলা হয়?</v>
       </c>
       <c r="B83" t="str">
-        <v>BTRI</v>
+        <v>ডোবা</v>
       </c>
       <c r="C83" t="str">
-        <v>BARI</v>
+        <v>হ্রদ</v>
       </c>
       <c r="D83" t="str">
-        <v>BRRI</v>
+        <v>বাঁওর</v>
       </c>
       <c r="E83" t="str">
-        <v>BADC</v>
+        <v>হাওর</v>
       </c>
       <c r="F83" t="str">
         <v>C</v>
@@ -2061,59 +2061,59 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>টমেটোকে উদ্যান ফসল বলার কারণ-</v>
+        <v>নিচের কোনটি দানা জাতীয় ফসল?</v>
       </c>
       <c r="B84" t="str">
-        <v>সমস্ত ফসল একত্রে সংগ্রহ করা হয়</v>
+        <v>ছোলা</v>
       </c>
       <c r="C84" t="str">
-        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
+        <v>সরিষা</v>
       </c>
       <c r="D84" t="str">
-        <v>নিচু ও মাঝারি নিচু জমিতে চাষ করা যায়</v>
+        <v>চীনা বাদাম</v>
       </c>
       <c r="E84" t="str">
-        <v>ফসলের দাম মৌসুমের শুরুতে কম থাকে</v>
+        <v>ধান</v>
       </c>
       <c r="F84" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয় কত সালে প্রতিষ্ঠিত হয় ?</v>
+        <v>BARI-এর প্রধান কার্যালয় কোথায়?</v>
       </c>
       <c r="B85" t="str">
-        <v>১৯৫৭</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="C85" t="str">
-        <v>১৯৬১</v>
+        <v>জামালপুর</v>
       </c>
       <c r="D85" t="str">
-        <v>১৯৬৫</v>
+        <v>ফরিদপুর</v>
       </c>
       <c r="E85" t="str">
-        <v>১৯৬৯</v>
+        <v>পিরোজপুর</v>
       </c>
       <c r="F85" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>পাটকে মাঠ ফসল বলার কারণ—</v>
+        <v>চাষাবাদে যন্ত্রশক্তির ব্যবহার কত?</v>
       </c>
       <c r="B86" t="str">
-        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
+        <v>৪০%</v>
       </c>
       <c r="C86" t="str">
-        <v>ফসলের লাভ ও ব্যয়ের অনুপাত বেশি হয়</v>
+        <v>৫০%</v>
       </c>
       <c r="D86" t="str">
-        <v>সমস্ত ফসল একত্রে পরিপক্ক ও সংগ্রহ করা হয়</v>
+        <v>৬০%</v>
       </c>
       <c r="E86" t="str">
-        <v>ফসলের মূল্য মৌসুমের শুরুতে বেশি হয়</v>
+        <v>৮০%</v>
       </c>
       <c r="F86" t="str">
         <v>C</v>
@@ -2121,99 +2121,99 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>নিচের কোনটি স্বাদু পানির মাছ?</v>
+        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
       </c>
       <c r="B87" t="str">
-        <v>রুপচান্দা</v>
+        <v>প্রতিটি গাছের আলাদাভাবে যত্ন নেওয়া হয়</v>
       </c>
       <c r="C87" t="str">
-        <v>ছুরি</v>
+        <v>জমির সমস্ত ফসল ধাপে ধাপে পরিপক্ক ও সংগ্রহ করতে হয়</v>
       </c>
       <c r="D87" t="str">
-        <v>পোয়া</v>
+        <v>মৌসুমের শুরুতে দাম কম থাকে পরবর্তীতে দাম বাড়ে</v>
       </c>
       <c r="E87" t="str">
-        <v>মাগুর</v>
+        <v>তুলনামূলকভাবে বেশি যত্নের প্রয়োজন হয়।</v>
       </c>
       <c r="F87" t="str">
-        <v>D</v>
+        <v>C</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>নিচের কোনটি মাঠ ফসল।</v>
+        <v>কোন প্রতিষ্ঠান কৃষকদের সার, বীজ কীটনাশক ও কৃষি যন্ত্রপাতি সরবরাহ করে?</v>
       </c>
       <c r="B88" t="str">
-        <v>পিঁয়াজ</v>
+        <v>BADC</v>
       </c>
       <c r="C88" t="str">
-        <v>ভুট্টা</v>
+        <v>BFDC</v>
       </c>
       <c r="D88" t="str">
-        <v>টমেটো</v>
+        <v>BARI</v>
       </c>
       <c r="E88" t="str">
-        <v>আম</v>
+        <v>BRRI</v>
       </c>
       <c r="F88" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা প্রতিষ্ঠান কত সালে প্রতিষ্ঠিত হয়?</v>
+        <v>নিচের কোনটি কৃষি সম্প্রসারণ প্রতিষ্ঠান।</v>
       </c>
       <c r="B89" t="str">
-        <v>১৯৭৪ সালে</v>
+        <v>DAE</v>
       </c>
       <c r="C89" t="str">
-        <v>১৯৭৬ সালে</v>
+        <v>BARI</v>
       </c>
       <c r="D89" t="str">
-        <v>১৯৭৮ সালে</v>
+        <v>BRRI</v>
       </c>
       <c r="E89" t="str">
-        <v>১৯৮০ সালে</v>
+        <v>BINA</v>
       </c>
       <c r="F89" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>নিচের কোনটি কৃষি গবেষণা প্রতিষ্ঠান?</v>
+        <v>নিচের কোন প্রতিষ্ঠানটি শুধুমাত্র ধান নিয়ে গবেষণা করে?</v>
       </c>
       <c r="B90" t="str">
-        <v>BAU</v>
+        <v>BARI</v>
       </c>
       <c r="C90" t="str">
+        <v>BINA</v>
+      </c>
+      <c r="D90" t="str">
         <v>BADC</v>
       </c>
-      <c r="D90" t="str">
-        <v>BARI</v>
-      </c>
       <c r="E90" t="str">
-        <v>SAU</v>
+        <v>BRRI</v>
       </c>
       <c r="F90" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>টমেটোকে উদ্যান ফসল বলার কারণ—</v>
+        <v>নিচের কোনটি কৃষি সম্প্রসারণ অধিদপ্তরের ওয়েবসাইট।</v>
       </c>
       <c r="B91" t="str">
-        <v>সমস্ত ফসল একত্রে সংগ্রহ করা হয়</v>
+        <v>www.ais.gov.bd</v>
       </c>
       <c r="C91" t="str">
-        <v>ফসলের নিবিড় যত্নের প্রয়োজন হয়</v>
+        <v>www.dae.gov.bd</v>
       </c>
       <c r="D91" t="str">
-        <v>নিচু ও মাঝারি নিচু জমিতে চাষ করা যায়</v>
+        <v>www.moa.gov.bd</v>
       </c>
       <c r="E91" t="str">
-        <v>ফসলের দাম মৌসুমের শুরুতে কম থাকে</v>
+        <v>www.brri.gov.bd</v>
       </c>
       <c r="F91" t="str">
         <v>B</v>
@@ -2221,19 +2221,19 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>কৃষি তথ্য সার্ভিসের সদর দপ্তর কোথায় অবস্থিত?</v>
+        <v>নিচের কোনটি দানা জাতীয় ফসল?</v>
       </c>
       <c r="B92" t="str">
-        <v>জয়দেবপুর</v>
+        <v>ছোলা</v>
       </c>
       <c r="C92" t="str">
-        <v>মহাখাল</v>
+        <v>সরিষা</v>
       </c>
       <c r="D92" t="str">
-        <v>ধানমণ্ডি</v>
+        <v>চীনাবাদাম</v>
       </c>
       <c r="E92" t="str">
-        <v>খামারবাড়ী</v>
+        <v>ধান</v>
       </c>
       <c r="F92" t="str">
         <v>D</v>
@@ -2241,199 +2241,199 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>নিচের কোনটি বদ্ধ জলাশয়ের উদাহরণ?</v>
+        <v>কোন উৎস থেকে কৃষক কৃষি বিষয়ক সকল তথ্য পেতে পারে?</v>
       </c>
       <c r="B93" t="str">
-        <v>নদী</v>
+        <v>উঠোন বৈঠক</v>
       </c>
       <c r="C93" t="str">
-        <v>খাল</v>
+        <v>কৃষিশিক্ষা বই</v>
       </c>
       <c r="D93" t="str">
-        <v>হাওর</v>
+        <v>এনজিও</v>
       </c>
       <c r="E93" t="str">
-        <v>বাঁওর</v>
+        <v>ইউনিয়ন সেবাকেন্দ্র</v>
       </c>
       <c r="F93" t="str">
-        <v>D</v>
+        <v>A</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>সর্বাধিক সংখ্যক কৃষি উপকরণ সরবরাহকারী প্রতিষ্ঠান কোনটি?</v>
+        <v>নিচের কোনটি উন্মুক্ত লোনা পানির মাছ?</v>
       </c>
       <c r="B94" t="str">
-        <v>বাংলাদেশ কৃষি বিশ্ববিদ্যালয়</v>
+        <v>ভেটকি</v>
       </c>
       <c r="C94" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট</v>
+        <v>বোয়াল</v>
       </c>
       <c r="D94" t="str">
-        <v>বাংলাদেশ ধান গবেষণা ইনস্টিটিউট</v>
+        <v>মৃগেল</v>
       </c>
       <c r="E94" t="str">
-        <v>বাংলাদেশ কৃষি উন্নয়ন কর্পোরেশন (BADC)</v>
+        <v>কার্পিও</v>
       </c>
       <c r="F94" t="str">
-        <v>D</v>
+        <v>A</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>নিচের কোনটি সবুজ সার জাতীয় ফসল?</v>
+        <v>গবেষণার জন্য বৈদেশিক সাহায্য আনয়নের ব্যবস্থা করে কোন প্রতিষ্ঠান?</v>
       </c>
       <c r="B95" t="str">
-        <v>চীনা</v>
+        <v>BARC</v>
       </c>
       <c r="C95" t="str">
-        <v>কফি</v>
+        <v>BADC</v>
       </c>
       <c r="D95" t="str">
-        <v>শণপাট</v>
+        <v>BARI</v>
       </c>
       <c r="E95" t="str">
-        <v>তিল</v>
+        <v>BRRI</v>
       </c>
       <c r="F95" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>কৃষি বন কোন বনায়নের অন্তর্ভুক্ত?</v>
+        <v>আন্তর্জাতিক ধান গবেষণা প্রতিষ্ঠানের সাথে মিল রয়েছে এমন একটি প্রতিষ্ঠান বাংলাদেশে আছে সেটির নাম কী?</v>
       </c>
       <c r="B96" t="str">
-        <v>সামাজিক বন</v>
+        <v>BTRI</v>
       </c>
       <c r="C96" t="str">
-        <v>সমতল বন</v>
+        <v>BARI</v>
       </c>
       <c r="D96" t="str">
-        <v>পাহাড়ি বন</v>
+        <v>BRRI</v>
       </c>
       <c r="E96" t="str">
-        <v>ম্যানগ্রোভ বন</v>
+        <v>BADC</v>
       </c>
       <c r="F96" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>নদীর প্রবাহ বাধাপ্রাপ্ত হয়ে উৎপন্ন জলাশয়কে কি বলা হয়?</v>
+        <v>বঙ্গবন্ধু শেখ মুজিবুর রহমান কৃষি বিশ্ববিদ্যালয়টি কোথায় অবস্থিত?</v>
       </c>
       <c r="B97" t="str">
-        <v>ডোবা</v>
+        <v>ঢাকা</v>
       </c>
       <c r="C97" t="str">
-        <v>হ্রদ</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="D97" t="str">
-        <v>বাঁওর</v>
+        <v>ময়মনসিংহ</v>
       </c>
       <c r="E97" t="str">
-        <v>হাওর</v>
+        <v>সিলেট</v>
       </c>
       <c r="F97" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>উঠোন বৈঠকের উদ্দেশ্য-</v>
+        <v>নতুন নতুন প্রযুক্তি সম্পর্কে খোজ খবর রাখেন কে?</v>
       </c>
       <c r="B98" t="str">
-        <v>অন্যায় থেকে বিরত রাখা</v>
+        <v>অভিজ্ঞ কৃষক</v>
       </c>
       <c r="C98" t="str">
-        <v>কৃষি তথ্য প্রচার করা</v>
+        <v>বয়স্ক কৃষক</v>
       </c>
       <c r="D98" t="str">
-        <v>স্কুলে যেতে উৎসাহ প্রদান</v>
+        <v>স্থানীয় মেম্বার</v>
       </c>
       <c r="E98" t="str">
-        <v>সবজির পুষ্টিগুণ প্রচার</v>
+        <v>স্কুল শিক্ষক</v>
       </c>
       <c r="F98" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>প্রাণিজগতকে কয়টি পর্বে ভাগ করা যায়?</v>
+        <v>স্থানীয় 'কৃষি তথ্য ভাণ্ডার' বলা হয় কাকে?</v>
       </c>
       <c r="B99" t="str">
-        <v>৮টি</v>
+        <v>সাধারণ কৃষক</v>
       </c>
       <c r="C99" t="str">
-        <v>৯টি</v>
+        <v>অভিজ্ঞ কৃষক</v>
       </c>
       <c r="D99" t="str">
-        <v>১০টি</v>
+        <v>বয়স্ক কৃষক</v>
       </c>
       <c r="E99" t="str">
-        <v>১১টি</v>
+        <v>কৃষক সভা</v>
       </c>
       <c r="F99" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট এর আঞ্চলিক কার্যালয় কয়টি?</v>
+        <v>ফসলের নতুন নতুন জাত উদ্ভাবন ও উন্নয়ন সাধনের কাজ করে নিচের কোন প্রতিষ্ঠানটি?</v>
       </c>
       <c r="B100" t="str">
-        <v>৩টি</v>
+        <v>BARI</v>
       </c>
       <c r="C100" t="str">
-        <v>৫টি</v>
+        <v>BINA</v>
       </c>
       <c r="D100" t="str">
-        <v>৬টি</v>
+        <v>BARC</v>
       </c>
       <c r="E100" t="str">
-        <v>৮টি</v>
+        <v>BRRI</v>
       </c>
       <c r="F100" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>নিচের কোনটি পানীয় ফসল?</v>
+        <v>কৃষক সভায় কতজন কৃষক অংশগ্রহণ করেন?</v>
       </c>
       <c r="B101" t="str">
-        <v>তামাক</v>
+        <v>১০-২০ জন</v>
       </c>
       <c r="C101" t="str">
-        <v>চা</v>
+        <v>৩০-৪০ জন</v>
       </c>
       <c r="D101" t="str">
-        <v>সরগম</v>
+        <v>৫০-৬০ জন</v>
       </c>
       <c r="E101" t="str">
-        <v>চিনা</v>
+        <v>৭০-৮০ জন</v>
       </c>
       <c r="F101" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>নিচের কোন প্রতিষ্ঠান কৃষক সভার আয়োজন করে?</v>
+        <v>হাতের স্পর্শের মাধ্যমে তথ্য প্রাপ্তির জন্য তৈরি করা হয়েছে কোনটি</v>
       </c>
       <c r="B102" t="str">
-        <v>কৃষি সম্প্রসারণ অধিদপ্তর</v>
+        <v>কিয়স্ক</v>
       </c>
       <c r="C102" t="str">
-        <v>বাংলাদেশ কৃষি উন্নয়ন কর্পোরেশন</v>
+        <v>কিমানো</v>
       </c>
       <c r="D102" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা কাউন্সিল</v>
+        <v>এস্কিমো</v>
       </c>
       <c r="E102" t="str">
-        <v>বাংলাদেশ কৃষি গবেষণা ইনস্টিটিউট</v>
+        <v>কিয়াটো</v>
       </c>
       <c r="F102" t="str">
         <v>A</v>
@@ -2441,79 +2441,79 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>নিচের কোন ফসলটি বেশি যত্নে চাষ করা হয়?</v>
+        <v>কৃষিতথ্য সার্ভিসের সদর দপ্তর কোথায় অবস্থিত?</v>
       </c>
       <c r="B103" t="str">
-        <v>গম</v>
+        <v>জয়দেবপুর</v>
       </c>
       <c r="C103" t="str">
-        <v>পাট</v>
+        <v>মহাখালী</v>
       </c>
       <c r="D103" t="str">
-        <v>টমেটো</v>
+        <v>ধানমণ্ডি</v>
       </c>
       <c r="E103" t="str">
-        <v>ইক্ষু</v>
+        <v>খামার বাড়ি</v>
       </c>
       <c r="F103" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>উদ্যান ফসলগুলো সাধারণত কত ভাগে বিভক্ত?</v>
+        <v>BRAC কত সালে প্রতিষ্ঠিত হয়?</v>
       </c>
       <c r="B104" t="str">
-        <v>২ ভাগে</v>
+        <v>১৯৭০</v>
       </c>
       <c r="C104" t="str">
-        <v>৩ ভাগে</v>
+        <v>১৯৭১</v>
       </c>
       <c r="D104" t="str">
-        <v>৪ ভাগে</v>
+        <v>১৯৭২</v>
       </c>
       <c r="E104" t="str">
-        <v>৫ ভাগে</v>
+        <v>১৯৭৩</v>
       </c>
       <c r="F104" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>কোনটি কনড্রিকথিস শ্রেণির মাছ?</v>
+        <v>নিচের কোনটি কৃষির তথ্য ও সেবা প্রাপ্তি প্রধান উৎস ?</v>
       </c>
       <c r="B105" t="str">
-        <v>কাতলা</v>
+        <v>অভিজ্ঞ কৃষক</v>
       </c>
       <c r="C105" t="str">
-        <v>হাঙ্গর</v>
+        <v>কৃষক সভা</v>
       </c>
       <c r="D105" t="str">
-        <v>তেলাপিয়া</v>
+        <v>কৃষক বিদ্যালয়সমূহ</v>
       </c>
       <c r="E105" t="str">
-        <v>কৈ</v>
+        <v>এনজিও</v>
       </c>
       <c r="F105" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>নিচের কোনটি কৃষির তথ্য ও সেবা প্রাপ্তি প্রধান উৎস ?</v>
+        <v>বাংলাদেশ পরমাণু কৃষি গবেষণা কোথায় অবস্থিত?</v>
       </c>
       <c r="B106" t="str">
-        <v>অভিজ্ঞ কৃষক</v>
+        <v>ময়মনসিংহ</v>
       </c>
       <c r="C106" t="str">
-        <v>কৃষক সভা</v>
+        <v>জামালপুর</v>
       </c>
       <c r="D106" t="str">
-        <v>কৃষক বিদ্যালয়সমূহ</v>
+        <v>জয়দেবপুর</v>
       </c>
       <c r="E106" t="str">
-        <v>এনজিও</v>
+        <v>হবিগঞ্জ</v>
       </c>
       <c r="F106" t="str">
         <v>A</v>
@@ -2521,59 +2521,59 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>কৃষিতথ্য সার্ভিসের সদর দপ্তর কোথায় অবস্থিত?</v>
+        <v>অভ্যন্তরীণ জলাশয়ের মধ্যে নিচের কোনটির আয়তন সবচেয়ে কম ?</v>
       </c>
       <c r="B107" t="str">
-        <v>জয়দেবপুর</v>
+        <v>পুকুর ডোবা</v>
       </c>
       <c r="C107" t="str">
-        <v>মহাখালী</v>
+        <v>বাঁওড়</v>
       </c>
       <c r="D107" t="str">
-        <v>ধানমন্ডি</v>
+        <v>বিল</v>
       </c>
       <c r="E107" t="str">
-        <v>খামার বাড়ি</v>
+        <v>চিংড়ি খামার</v>
       </c>
       <c r="F107" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>বাউকুলের উদ্ভাবক প্রতিষ্ঠান কোনটি?</v>
+        <v>বাংলাদেশে কৃষি গবেষণা কাউন্সিল প্রতিষ্ঠিত হয় কত সালে?</v>
       </c>
       <c r="B108" t="str">
-        <v>বা.কৃ.বি.</v>
+        <v>১৯৭১ সালে</v>
       </c>
       <c r="C108" t="str">
-        <v>শে.কৃ.বি.</v>
+        <v>১৯৭২ সালে</v>
       </c>
       <c r="D108" t="str">
-        <v>বারি</v>
+        <v>১৯৭৩ সালে</v>
       </c>
       <c r="E108" t="str">
-        <v>বিজেআরআই</v>
+        <v>১৯৭৪ সালে</v>
       </c>
       <c r="F108" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>নিচের কোনটি উন্মুক্ত লোনা পানির মাছ?</v>
+        <v>বাংলাদেশ পাট গবেষণা ইনস্টিটিউট কোথায় অবস্থিত?</v>
       </c>
       <c r="B109" t="str">
-        <v>ভেটকি</v>
+        <v>ঢাকা</v>
       </c>
       <c r="C109" t="str">
-        <v>বোয়াল</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="D109" t="str">
-        <v>মৃগেল</v>
+        <v>টাঙ্গাইল</v>
       </c>
       <c r="E109" t="str">
-        <v>কার্পিও</v>
+        <v>পাবনা</v>
       </c>
       <c r="F109" t="str">
         <v>A</v>
@@ -2581,62 +2581,62 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>পোল্ট্রি কোনটি?</v>
+        <v>কৃষি তথ্যের সবচেয়ে বড় ভাণ্ডার কোনটি?</v>
       </c>
       <c r="B110" t="str">
-        <v>টিয়া</v>
+        <v>কৃষি কথা পত্রিকা</v>
       </c>
       <c r="C110" t="str">
-        <v>টার্কি</v>
+        <v>মোবাইল ফোন</v>
       </c>
       <c r="D110" t="str">
-        <v>ময়না</v>
+        <v>টেলিভিশন</v>
       </c>
       <c r="E110" t="str">
-        <v>ঘুঘু</v>
+        <v>ইন্টারনেট</v>
       </c>
       <c r="F110" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>প্রাণিজ আমিষের প্রায় কত ভাগ মাছ থেকে আসে?</v>
+        <v>BRRI এর প্রধান কার্যালয় কোথায় ?</v>
       </c>
       <c r="B111" t="str">
-        <v>৪০%</v>
+        <v>রাজশাহী</v>
       </c>
       <c r="C111" t="str">
-        <v>৫০%</v>
+        <v>দিনাজপুর</v>
       </c>
       <c r="D111" t="str">
-        <v>৬০%</v>
+        <v>ময়মনসিংহ</v>
       </c>
       <c r="E111" t="str">
-        <v>৭০%</v>
+        <v>গাজীপুর</v>
       </c>
       <c r="F111" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>কৃষির প্রধান ক্ষেত্র-</v>
+        <v>কৃষি উপকরণ সরবরাহকারী সরকারি প্রতিষ্ঠান কোনটি?</v>
       </c>
       <c r="B112" t="str">
-        <v>২ টি</v>
+        <v>বিএডিসি</v>
       </c>
       <c r="C112" t="str">
-        <v>৪ টি</v>
+        <v>কৃষি তথ্য সার্ভিস</v>
       </c>
       <c r="D112" t="str">
-        <v>৬ টি</v>
+        <v>ডি এই</v>
       </c>
       <c r="E112" t="str">
-        <v>৮ টি</v>
+        <v>বি আর আই</v>
       </c>
       <c r="F112" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>